<commit_message>
Republish AMR to the website
Surfaces regenerated (sitemap/footer, feed, market registry, chart + technicals); freshness and page-integrity gates clean; verified by headless render.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/AMR_Valuation_Model_09082026.xlsx
+++ b/files/AMR_Valuation_Model_09082026.xlsx
@@ -2575,111 +2575,111 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>8.00%</t>
+          <t>8.20%</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>2.689963203325789</v>
+        <v>2.59881486006034</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2.860337885054136</v>
+        <v>2.75578000679716</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>3.064248697728378</v>
+        <v>2.942432946714026</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>3.312848422877485</v>
+        <v>3.168230612770638</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>3.622851685899725</v>
+        <v>3.447123723786802</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>8.75%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>2.362314109361936</v>
+        <v>2.29037370929778</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2.488118720415106</v>
+        <v>2.407165738467058</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>2.635369723229186</v>
+        <v>2.54318052228866</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>2.810182471952523</v>
+        <v>2.703700107790479</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>3.021241547941936</v>
+        <v>2.896136874934558</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>2.100325927119413</v>
+        <v>2.042163821293314</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>2.195715870481494</v>
+        <v>2.131257662042504</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>2.305421681630923</v>
+        <v>2.233308017752015</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>2.433016097897558</v>
+        <v>2.351445039158722</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>2.583368567260923</v>
+        <v>2.489895464546122</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>10.25%</t>
+          <t>10.45%</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1.886105952820147</v>
+        <v>1.838156556980712</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>1.959982266853094</v>
+        <v>1.907495924832088</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>2.043742616089398</v>
+        <v>1.985850313836771</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>2.13958005375153</v>
+        <v>2.075162925425672</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>2.250388237346297</v>
+        <v>2.177978674447895</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>1.707719127700286</v>
+        <v>1.667545283529673</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>1.765930588738839</v>
+        <v>1.722403267209278</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>1.831153911590974</v>
+        <v>1.783697011530936</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1.90478951514285</v>
+        <v>1.852678789731079</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>1.988637340851779</v>
+        <v>1.930948299583152</v>
       </c>
     </row>
     <row r="12">
@@ -2719,111 +2719,111 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>8.00%</t>
+          <t>8.20%</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>2.596476620793644</v>
+        <v>2.491868709377671</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>2.83036265926101</v>
+        <v>2.717150828045848</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>3.064248697728378</v>
+        <v>2.942432946714026</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>3.298134736195744</v>
+        <v>3.167715065382204</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>3.532020774663111</v>
+        <v>3.392997184050382</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>8.75%</t>
+          <t>8.95%</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>2.22829044897828</v>
+        <v>2.149127751906584</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>2.431830086103732</v>
+        <v>2.346154137097622</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>2.635369723229186</v>
+        <v>2.54318052228866</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>2.838909360354638</v>
+        <v>2.740206907479699</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>3.04244899748009</v>
+        <v>2.937233292670737</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>9.50%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>1.945071282019615</v>
+        <v>1.883150389198714</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>2.125246481825268</v>
+        <v>2.058229203475364</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>2.305421681630923</v>
+        <v>2.233308017752015</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>2.485596881436576</v>
+        <v>2.408386832028666</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>2.665772081242229</v>
+        <v>2.583465646305317</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>10.25%</t>
+          <t>10.45%</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>1.720483475001578</v>
+        <v>1.670776226627332</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>1.882113045545488</v>
+        <v>1.828313270232051</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>2.043742616089398</v>
+        <v>1.985850313836771</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>2.205372186633307</v>
+        <v>2.14338735744149</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>2.367001757177217</v>
+        <v>2.30092440104621</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>11.00%</t>
+          <t>11.20%</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>1.538054535967304</v>
+        <v>1.497309182309147</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>1.684604223779139</v>
+        <v>1.640503096920041</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>1.831153911590974</v>
+        <v>1.783697011530936</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>1.977703599402809</v>
+        <v>1.926890926141831</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>2.124253287214644</v>
+        <v>2.070084840752726</v>
       </c>
     </row>
     <row r="20">
@@ -2845,19 +2845,19 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>2.15658397818916</v>
+        <v>2.089254026961081</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>2.230264896942197</v>
+        <v>2.160567950500811</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>2.305421681630923</v>
+        <v>2.233308017752015</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>2.38207632785189</v>
+        <v>2.307495465459392</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>2.460251047727809</v>
+        <v>2.383151739324826</v>
       </c>
       <c r="H21" s="12">
         <f>MAX(B21:F21)-MIN(B21:F21)</f>
@@ -2871,19 +2871,19 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>1.945071282019615</v>
+        <v>1.883150389198714</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>2.125246481825268</v>
+        <v>2.058229203475364</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>2.305421681630923</v>
+        <v>2.233308017752015</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>2.485596881436576</v>
+        <v>2.408386832028666</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>2.665772081242229</v>
+        <v>2.583465646305317</v>
       </c>
       <c r="H22" s="12">
         <f>MAX(B22:F22)-MIN(B22:F22)</f>
@@ -2897,19 +2897,19 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>3.064248697728378</v>
+        <v>2.942432946714026</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>2.635369723229186</v>
+        <v>2.54318052228866</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>2.305421681630923</v>
+        <v>2.233308017752015</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>2.043742616089398</v>
+        <v>1.985850313836771</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>1.831153911590974</v>
+        <v>1.783697011530936</v>
       </c>
       <c r="H23" s="12">
         <f>MAX(B23:F23)-MIN(B23:F23)</f>
@@ -2923,19 +2923,19 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>2.100325927119413</v>
+        <v>2.042163821293314</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>2.195715870481494</v>
+        <v>2.131257662042504</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>2.305421681630923</v>
+        <v>2.233308017752015</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>2.433016097897558</v>
+        <v>2.351445039158722</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>2.583368567260923</v>
+        <v>2.489895464546122</v>
       </c>
       <c r="H24" s="12">
         <f>MAX(B24:F24)-MIN(B24:F24)</f>
@@ -4102,14 +4102,14 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>1.400021011084784</v>
+        <v>1.366554912808877</v>
       </c>
       <c r="C5" s="10">
         <f>DCF!C39</f>
         <v/>
       </c>
       <c r="D5" s="9" t="n">
-        <v>4.29768913036704</v>
+        <v>4.090210014429833</v>
       </c>
       <c r="E5" s="11">
         <f>Assumptions!$C$103</f>
@@ -4674,7 +4674,7 @@
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>2.305421681630923</v>
+        <v>2.233308017752015</v>
       </c>
     </row>
     <row r="20">
@@ -4684,7 +4684,7 @@
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>2.259144982128687</v>
+        <v>2.195924444939009</v>
       </c>
     </row>
     <row r="21">
@@ -5695,7 +5695,7 @@
         </is>
       </c>
       <c r="C81" s="18" t="n">
-        <v>0.894</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="82">

</xml_diff>